<commit_message>
feat: add 04_pipeline_testing notebook (pipeline testing minggu 4)
</commit_message>
<xml_diff>
--- a/reports/rekap_15_model.xlsx
+++ b/reports/rekap_15_model.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,31 +512,31 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7071</v>
+        <v>0.7272</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9579</v>
+        <v>0.9702</v>
       </c>
       <c r="F2" t="n">
-        <v>0.998</v>
+        <v>0.9978</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7997</v>
+        <v>0.7309</v>
       </c>
       <c r="H2" t="n">
-        <v>1.0419</v>
+        <v>0.9533</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9979</v>
+        <v>0.9981</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7071</v>
+        <v>0.7272</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9579</v>
+        <v>0.9702</v>
       </c>
       <c r="L2" t="n">
-        <v>0.998</v>
+        <v>0.9978</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -561,31 +561,31 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7257</v>
+        <v>0.7433</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0061</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9979</v>
+        <v>0.9977</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8276</v>
+        <v>0.734</v>
       </c>
       <c r="H3" t="n">
-        <v>1.0697</v>
+        <v>0.978</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9978</v>
+        <v>0.998</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7257</v>
+        <v>0.734</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9874000000000001</v>
+        <v>0.978</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9979</v>
+        <v>0.998</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -606,35 +606,35 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LGBMRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.1687</v>
+        <v>0.1555</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2361</v>
+        <v>0.2177</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8315</v>
+        <v>0.8602</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2074</v>
+        <v>1.1555</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2843</v>
+        <v>0.2177</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7582</v>
+        <v>0.8602</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1687</v>
+        <v>0.1555</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2361</v>
+        <v>0.2177</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8315</v>
+        <v>0.8602</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -655,35 +655,35 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LGBMRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3.5041</v>
+        <v>3.2171</v>
       </c>
       <c r="E5" t="n">
-        <v>4.9069</v>
+        <v>4.4011</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9008</v>
+        <v>0.9176</v>
       </c>
       <c r="G5" t="n">
-        <v>4.2378</v>
+        <v>4.2171</v>
       </c>
       <c r="H5" t="n">
-        <v>6.3573</v>
+        <v>4.4011</v>
       </c>
       <c r="I5" t="n">
-        <v>0.846</v>
+        <v>0.9176</v>
       </c>
       <c r="J5" t="n">
-        <v>3.5041</v>
+        <v>3.2171</v>
       </c>
       <c r="K5" t="n">
-        <v>4.9069</v>
+        <v>4.4011</v>
       </c>
       <c r="L5" t="n">
-        <v>0.9008</v>
+        <v>0.9176</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -704,35 +704,35 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LGBMRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11.5384</v>
+        <v>10.5413</v>
       </c>
       <c r="E6" t="n">
-        <v>15.2594</v>
+        <v>13.8503</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8871</v>
+        <v>0.905</v>
       </c>
       <c r="G6" t="n">
-        <v>11.8563</v>
+        <v>11.5413</v>
       </c>
       <c r="H6" t="n">
-        <v>14.9884</v>
+        <v>13.8503</v>
       </c>
       <c r="I6" t="n">
-        <v>0.875</v>
+        <v>0.905</v>
       </c>
       <c r="J6" t="n">
-        <v>11.5384</v>
+        <v>10.5413</v>
       </c>
       <c r="K6" t="n">
-        <v>15.2594</v>
+        <v>13.8503</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8871</v>
+        <v>0.905</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -757,31 +757,31 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.3534</v>
+        <v>0.372</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4879</v>
+        <v>0.5143</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9974</v>
+        <v>0.997</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3563</v>
+        <v>0.3801</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5219</v>
+        <v>0.5223</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9973</v>
+        <v>0.9976</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3534</v>
+        <v>0.372</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4879</v>
+        <v>0.5143</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9974</v>
+        <v>0.997</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -806,31 +806,31 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3718</v>
+        <v>0.3859</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5127</v>
+        <v>0.5374</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9972</v>
+        <v>0.9968</v>
       </c>
       <c r="G8" t="n">
-        <v>0.377</v>
+        <v>0.3832</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5416</v>
+        <v>0.541</v>
       </c>
       <c r="I8" t="n">
-        <v>0.9972</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3718</v>
+        <v>0.3832</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5127</v>
+        <v>0.541</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9972</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -851,35 +851,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LGBMRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.1465</v>
+        <v>0.1345</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1963</v>
+        <v>0.187</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8345</v>
+        <v>0.8442</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1626</v>
+        <v>1.1345</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2104</v>
+        <v>0.187</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8288</v>
+        <v>0.8442</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1465</v>
+        <v>0.1345</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1963</v>
+        <v>0.187</v>
       </c>
       <c r="L9" t="n">
-        <v>0.8345</v>
+        <v>0.8442</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -900,35 +900,35 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ExtraTreesRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.6263</v>
+        <v>2.2503</v>
       </c>
       <c r="E10" t="n">
-        <v>3.0691</v>
+        <v>3.2758</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6528</v>
+        <v>0.8581</v>
       </c>
       <c r="G10" t="n">
-        <v>3.2136</v>
+        <v>3.2503</v>
       </c>
       <c r="H10" t="n">
-        <v>4.7661</v>
+        <v>3.2758</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7821</v>
+        <v>0.8581</v>
       </c>
       <c r="J10" t="n">
-        <v>1.6263</v>
+        <v>2.2503</v>
       </c>
       <c r="K10" t="n">
-        <v>3.0691</v>
+        <v>3.2758</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6528</v>
+        <v>0.8581</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -949,35 +949,35 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LGBMRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>12.8673</v>
+        <v>11.6033</v>
       </c>
       <c r="E11" t="n">
-        <v>16.8834</v>
+        <v>15.1596</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8253</v>
+        <v>0.8673999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>13.5881</v>
+        <v>12.6033</v>
       </c>
       <c r="H11" t="n">
-        <v>18.1284</v>
+        <v>15.1596</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8028999999999999</v>
+        <v>0.8673999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>12.8673</v>
+        <v>11.6033</v>
       </c>
       <c r="K11" t="n">
-        <v>16.8834</v>
+        <v>15.1596</v>
       </c>
       <c r="L11" t="n">
-        <v>0.8253</v>
+        <v>0.8673999999999999</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -998,35 +998,35 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BayesianRidge</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5387999999999999</v>
+        <v>0.5459000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7192</v>
+        <v>0.7356</v>
       </c>
       <c r="F12" t="n">
+        <v>0.9988</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.5204</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.6937</v>
+      </c>
+      <c r="I12" t="n">
         <v>0.9989</v>
       </c>
-      <c r="G12" t="n">
-        <v>0.5088</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.6522</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.9988</v>
-      </c>
       <c r="J12" t="n">
-        <v>0.5088</v>
+        <v>0.5204</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6522</v>
+        <v>0.6937</v>
       </c>
       <c r="L12" t="n">
-        <v>0.9988</v>
+        <v>0.9989</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1051,28 +1051,28 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.5343</v>
+        <v>0.5417</v>
       </c>
       <c r="E13" t="n">
-        <v>0.716</v>
+        <v>0.733</v>
       </c>
       <c r="F13" t="n">
         <v>0.9989</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5057</v>
+        <v>0.519</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6465</v>
+        <v>0.6938</v>
       </c>
       <c r="I13" t="n">
         <v>0.9989</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5057</v>
+        <v>0.519</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6465</v>
+        <v>0.6938</v>
       </c>
       <c r="L13" t="n">
         <v>0.9989</v>
@@ -1096,35 +1096,35 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ExtraTreesRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.2583</v>
+        <v>0.2301</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3512</v>
+        <v>0.3112</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8327</v>
+        <v>0.8633</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3864</v>
+        <v>1.2301</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4817</v>
+        <v>0.3112</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6767</v>
+        <v>0.8633</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2583</v>
+        <v>0.2301</v>
       </c>
       <c r="K14" t="n">
-        <v>0.3512</v>
+        <v>0.3112</v>
       </c>
       <c r="L14" t="n">
-        <v>0.8327</v>
+        <v>0.8633</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1145,35 +1145,35 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ExtraTreesRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3.9661</v>
+        <v>3.2531</v>
       </c>
       <c r="E15" t="n">
-        <v>5.878</v>
+        <v>5.0616</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9084</v>
+        <v>0.9304</v>
       </c>
       <c r="G15" t="n">
-        <v>4.9615</v>
+        <v>4.2531</v>
       </c>
       <c r="H15" t="n">
-        <v>6.6105</v>
+        <v>5.0616</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8118</v>
+        <v>0.9304</v>
       </c>
       <c r="J15" t="n">
-        <v>3.9661</v>
+        <v>3.2531</v>
       </c>
       <c r="K15" t="n">
-        <v>5.878</v>
+        <v>5.0616</v>
       </c>
       <c r="L15" t="n">
-        <v>0.9084</v>
+        <v>0.9304</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1194,35 +1194,35 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ExtraTreesRegressor</t>
+          <t>CatBoostRegressor</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6.3425</v>
+        <v>5.4484</v>
       </c>
       <c r="E16" t="n">
-        <v>8.9055</v>
+        <v>7.7429</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8238</v>
+        <v>0.8672</v>
       </c>
       <c r="G16" t="n">
-        <v>9.560600000000001</v>
+        <v>6.4484</v>
       </c>
       <c r="H16" t="n">
-        <v>12.6698</v>
+        <v>7.7429</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6729000000000001</v>
+        <v>0.8672</v>
       </c>
       <c r="J16" t="n">
-        <v>6.3425</v>
+        <v>5.4484</v>
       </c>
       <c r="K16" t="n">
-        <v>8.9055</v>
+        <v>7.7429</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8238</v>
+        <v>0.8672</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: finalisasi semua notebook, perbaikan time series validation, pipeline testing, dan visualisasi slide
</commit_message>
<xml_diff>
--- a/reports/rekap_15_model.xlsx
+++ b/reports/rekap_15_model.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -508,35 +508,35 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BayesianRidge</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7272</v>
+        <v>0.8525</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9702</v>
+        <v>1.1143</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9978</v>
+        <v>0.9948</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7309</v>
+        <v>1.0366</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9533</v>
+        <v>1.4168</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9981</v>
+        <v>0.9834000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7272</v>
+        <v>0.8525</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9702</v>
+        <v>1.1143</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9978</v>
+        <v>0.9948</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -557,35 +557,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BayesianRidge</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7433</v>
+        <v>0.895</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0061</v>
+        <v>1.1619</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9977</v>
+        <v>0.9933999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>0.734</v>
+        <v>1.1486</v>
       </c>
       <c r="H3" t="n">
-        <v>0.978</v>
+        <v>1.5673</v>
       </c>
       <c r="I3" t="n">
-        <v>0.998</v>
+        <v>0.9792999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>0.734</v>
+        <v>0.895</v>
       </c>
       <c r="K3" t="n">
-        <v>0.978</v>
+        <v>1.1619</v>
       </c>
       <c r="L3" t="n">
-        <v>0.998</v>
+        <v>0.9933999999999999</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -606,35 +606,35 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>ExtraTreesRegressor</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.1555</v>
+        <v>0.2245</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2177</v>
+        <v>0.2868</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8602</v>
+        <v>0.6733</v>
       </c>
       <c r="G4" t="n">
-        <v>1.1555</v>
+        <v>0.1594</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2177</v>
+        <v>0.1978</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8602</v>
+        <v>0.718</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1555</v>
+        <v>0.1594</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2177</v>
+        <v>0.1978</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8602</v>
+        <v>0.718</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -655,35 +655,35 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>LGBMRegressor</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3.2171</v>
+        <v>4.5483</v>
       </c>
       <c r="E5" t="n">
-        <v>4.4011</v>
+        <v>5.8697</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9176</v>
+        <v>0.796</v>
       </c>
       <c r="G5" t="n">
-        <v>4.2171</v>
+        <v>3.2362</v>
       </c>
       <c r="H5" t="n">
-        <v>4.4011</v>
+        <v>4.0677</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9176</v>
+        <v>0.7595</v>
       </c>
       <c r="J5" t="n">
-        <v>3.2171</v>
+        <v>3.2362</v>
       </c>
       <c r="K5" t="n">
-        <v>4.4011</v>
+        <v>4.0677</v>
       </c>
       <c r="L5" t="n">
-        <v>0.9176</v>
+        <v>0.7595</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -704,35 +704,35 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>ExtraTreesRegressor</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.5413</v>
+        <v>14.8967</v>
       </c>
       <c r="E6" t="n">
-        <v>13.8503</v>
+        <v>19.2176</v>
       </c>
       <c r="F6" t="n">
-        <v>0.905</v>
+        <v>0.8147</v>
       </c>
       <c r="G6" t="n">
-        <v>11.5413</v>
+        <v>17.6389</v>
       </c>
       <c r="H6" t="n">
-        <v>13.8503</v>
+        <v>22.0183</v>
       </c>
       <c r="I6" t="n">
-        <v>0.905</v>
+        <v>0.7443</v>
       </c>
       <c r="J6" t="n">
-        <v>10.5413</v>
+        <v>14.8967</v>
       </c>
       <c r="K6" t="n">
-        <v>13.8503</v>
+        <v>19.2176</v>
       </c>
       <c r="L6" t="n">
-        <v>0.905</v>
+        <v>0.8147</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -757,31 +757,31 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.372</v>
+        <v>0.578</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5143</v>
+        <v>0.7674</v>
       </c>
       <c r="F7" t="n">
-        <v>0.997</v>
+        <v>0.987</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3801</v>
+        <v>0.6332</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5223</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9976</v>
+        <v>0.9764</v>
       </c>
       <c r="J7" t="n">
-        <v>0.372</v>
+        <v>0.578</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5143</v>
+        <v>0.7674</v>
       </c>
       <c r="L7" t="n">
-        <v>0.997</v>
+        <v>0.987</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -806,31 +806,31 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3859</v>
+        <v>0.5654</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5374</v>
+        <v>0.7594</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9968</v>
+        <v>0.9867</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3832</v>
+        <v>0.6254999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.541</v>
+        <v>0.8861</v>
       </c>
       <c r="I8" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9752</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3832</v>
+        <v>0.5654</v>
       </c>
       <c r="K8" t="n">
-        <v>0.541</v>
+        <v>0.7594</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9867</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -851,35 +851,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>GradientBoostingRegressor</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.1345</v>
+        <v>0.1978</v>
       </c>
       <c r="E9" t="n">
-        <v>0.187</v>
+        <v>0.257</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8442</v>
+        <v>0.6034</v>
       </c>
       <c r="G9" t="n">
-        <v>1.1345</v>
+        <v>0.1515</v>
       </c>
       <c r="H9" t="n">
-        <v>0.187</v>
+        <v>0.2057</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8442</v>
+        <v>0.7105</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1345</v>
+        <v>0.1515</v>
       </c>
       <c r="K9" t="n">
-        <v>0.187</v>
+        <v>0.2057</v>
       </c>
       <c r="L9" t="n">
-        <v>0.8442</v>
+        <v>0.7105</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -900,35 +900,35 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>LGBMRegressor</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.2503</v>
+        <v>3.0296</v>
       </c>
       <c r="E10" t="n">
-        <v>3.2758</v>
+        <v>4.0863</v>
       </c>
       <c r="F10" t="n">
-        <v>0.8581</v>
+        <v>0.7619</v>
       </c>
       <c r="G10" t="n">
-        <v>3.2503</v>
+        <v>3.0341</v>
       </c>
       <c r="H10" t="n">
-        <v>3.2758</v>
+        <v>3.8935</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8581</v>
+        <v>0.749</v>
       </c>
       <c r="J10" t="n">
-        <v>2.2503</v>
+        <v>3.0296</v>
       </c>
       <c r="K10" t="n">
-        <v>3.2758</v>
+        <v>4.0863</v>
       </c>
       <c r="L10" t="n">
-        <v>0.8581</v>
+        <v>0.7619</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -949,35 +949,35 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>BayesianRidge</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>11.6033</v>
+        <v>18.4591</v>
       </c>
       <c r="E11" t="n">
-        <v>15.1596</v>
+        <v>23.0501</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8673999999999999</v>
+        <v>0.6109</v>
       </c>
       <c r="G11" t="n">
-        <v>12.6033</v>
+        <v>11.3752</v>
       </c>
       <c r="H11" t="n">
-        <v>15.1596</v>
+        <v>16.5023</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8673999999999999</v>
+        <v>0.7584</v>
       </c>
       <c r="J11" t="n">
-        <v>11.6033</v>
+        <v>11.3752</v>
       </c>
       <c r="K11" t="n">
-        <v>15.1596</v>
+        <v>16.5023</v>
       </c>
       <c r="L11" t="n">
-        <v>0.8673999999999999</v>
+        <v>0.7584</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -998,35 +998,35 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.592</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7356</v>
+        <v>0.8208</v>
       </c>
       <c r="F12" t="n">
-        <v>0.9988</v>
+        <v>0.9969</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5204</v>
+        <v>0.6774</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6937</v>
+        <v>0.9176</v>
       </c>
       <c r="I12" t="n">
-        <v>0.9989</v>
+        <v>0.9918</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5204</v>
+        <v>0.592</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6937</v>
+        <v>0.8208</v>
       </c>
       <c r="L12" t="n">
-        <v>0.9989</v>
+        <v>0.9969</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1047,35 +1047,35 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BayesianRidge</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.5417</v>
+        <v>0.55</v>
       </c>
       <c r="E13" t="n">
-        <v>0.733</v>
+        <v>0.7452</v>
       </c>
       <c r="F13" t="n">
-        <v>0.9989</v>
+        <v>0.9973</v>
       </c>
       <c r="G13" t="n">
-        <v>0.519</v>
+        <v>0.6545</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6938</v>
+        <v>0.884</v>
       </c>
       <c r="I13" t="n">
-        <v>0.9989</v>
+        <v>0.992</v>
       </c>
       <c r="J13" t="n">
-        <v>0.519</v>
+        <v>0.55</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6938</v>
+        <v>0.7452</v>
       </c>
       <c r="L13" t="n">
-        <v>0.9989</v>
+        <v>0.9973</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1096,35 +1096,35 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>LGBMRegressor</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.2301</v>
+        <v>0.3681</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3112</v>
+        <v>0.467</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8633</v>
+        <v>0.5641</v>
       </c>
       <c r="G14" t="n">
-        <v>1.2301</v>
+        <v>0.232</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3112</v>
+        <v>0.3053</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8633</v>
+        <v>0.7916</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2301</v>
+        <v>0.232</v>
       </c>
       <c r="K14" t="n">
-        <v>0.3112</v>
+        <v>0.3053</v>
       </c>
       <c r="L14" t="n">
-        <v>0.8633</v>
+        <v>0.7916</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1145,35 +1145,35 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3.2531</v>
+        <v>5.4393</v>
       </c>
       <c r="E15" t="n">
-        <v>5.0616</v>
+        <v>7.6449</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9304</v>
+        <v>0.764</v>
       </c>
       <c r="G15" t="n">
-        <v>4.2531</v>
+        <v>3.9894</v>
       </c>
       <c r="H15" t="n">
-        <v>5.0616</v>
+        <v>5.0328</v>
       </c>
       <c r="I15" t="n">
-        <v>0.9304</v>
+        <v>0.7817</v>
       </c>
       <c r="J15" t="n">
-        <v>3.2531</v>
+        <v>3.9894</v>
       </c>
       <c r="K15" t="n">
-        <v>5.0616</v>
+        <v>5.0328</v>
       </c>
       <c r="L15" t="n">
-        <v>0.9304</v>
+        <v>0.7817</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1194,35 +1194,35 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CatBoostRegressor</t>
+          <t>GradientBoostingRegressor</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5.4484</v>
+        <v>10.6034</v>
       </c>
       <c r="E16" t="n">
-        <v>7.7429</v>
+        <v>13.9629</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8672</v>
+        <v>0.5508</v>
       </c>
       <c r="G16" t="n">
-        <v>6.4484</v>
+        <v>12.0921</v>
       </c>
       <c r="H16" t="n">
-        <v>7.7429</v>
+        <v>15.9515</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8672</v>
+        <v>0.3565</v>
       </c>
       <c r="J16" t="n">
-        <v>5.4484</v>
+        <v>10.6034</v>
       </c>
       <c r="K16" t="n">
-        <v>7.7429</v>
+        <v>13.9629</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8672</v>
+        <v>0.5508</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>

</xml_diff>